<commit_message>
v5.1 istanbul samsun eklendi - tramvay km ve bakim plani sayfaları eklendi
</commit_message>
<xml_diff>
--- a/data/istanbul/Veriler.xlsx
+++ b/data/istanbul/Veriler.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fatiherkin\Desktop\bozankaya_ssh_takip\data\istanbul\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD9629ED-43E8-4766-BE00-2D43233EA738}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC1E5A9F-FABF-4A15-8D74-B7AE115C94B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="768" yWindow="768" windowWidth="17280" windowHeight="9960" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1920" yWindow="1920" windowWidth="17280" windowHeight="9960" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sayfa1" sheetId="1" r:id="rId1"/>
@@ -2368,7 +2368,7 @@
     </row>
     <row r="2" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1">
-        <v>1</v>
+        <v>9001</v>
       </c>
       <c r="B2" t="s">
         <v>199</v>
@@ -2391,7 +2391,7 @@
     </row>
     <row r="3" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="1">
-        <v>2</v>
+        <v>9002</v>
       </c>
       <c r="B3" t="s">
         <v>200</v>
@@ -2411,7 +2411,7 @@
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" s="1">
-        <v>3</v>
+        <v>9003</v>
       </c>
       <c r="C4" t="s">
         <v>190</v>
@@ -2428,7 +2428,7 @@
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" s="1">
-        <v>4</v>
+        <v>9004</v>
       </c>
       <c r="C5" t="s">
         <v>194</v>
@@ -2439,36 +2439,26 @@
     </row>
     <row r="6" spans="1:7" ht="27" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="1">
-        <v>5</v>
+        <v>9005</v>
       </c>
       <c r="C6" t="s">
         <v>196</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="27" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="1">
-        <v>6</v>
-      </c>
+      <c r="A7" s="1"/>
     </row>
     <row r="8" spans="1:7" ht="27" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="1">
-        <v>7</v>
-      </c>
+      <c r="A8" s="1"/>
     </row>
     <row r="9" spans="1:7" ht="27" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="1">
-        <v>8</v>
-      </c>
+      <c r="A9" s="1"/>
     </row>
     <row r="10" spans="1:7" ht="27" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="1">
-        <v>9</v>
-      </c>
+      <c r="A10" s="1"/>
     </row>
     <row r="11" spans="1:7" ht="27" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="1">
-        <v>10</v>
-      </c>
+      <c r="A11" s="1"/>
     </row>
     <row r="12" spans="1:7" ht="27" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="1"/>

</xml_diff>